<commit_message>
Match real workbook layout; add configurable date format
- System name now comes solely from the tab name; in-sheet "System" column
  is ignored. Recognise "Holiday Ccy" / "Holiday Date" headers.
- Add --date-format (default MM/DD/YYYY) for parsing text dates and report
  output; exposed as a workflow_dispatch input.
- Update sample generator, demo data, and README to real layout
  (System | Holiday Ccy | Holiday Date; tabs WSS/Barracuda/Broadway/D3).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/holidays.xlsx
+++ b/input/holidays.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="D3" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Barracuda" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="WSS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Barracuda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Broadway" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="D3" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,16 +416,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
+        <is>
+          <t>Holiday Ccy</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>Holiday Date</t>
         </is>
@@ -433,84 +439,119 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>WSS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01/01/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>WSS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>07/01/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>02/16/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>WSS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>12/25/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>WSS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>WSS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07/04/2020</t>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HKD</t>
+          <t>WSS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HKD</t>
+          <t>WSS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10/01/2020</t>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>08/17/2026</t>
         </is>
       </c>
     </row>
@@ -525,16 +566,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
+        <is>
+          <t>Holiday Ccy</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>Holiday Date</t>
         </is>
@@ -543,84 +589,119 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>Barracuda</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01/01/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>Barracuda</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>07/01/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>02/16/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Barracuda</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Barracuda</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>07/04/2020</t>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Barracuda</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>11/26/2020</t>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HKD</t>
+          <t>Barracuda</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>08/17/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HKD</t>
+          <t>Barracuda</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10/01/2020</t>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>08/17/2026</t>
         </is>
       </c>
     </row>
@@ -635,16 +716,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
+        <is>
+          <t>Holiday Ccy</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>Holiday Date</t>
         </is>
@@ -653,60 +739,218 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>Broadway</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01/01/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>Broadway</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>07/01/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>02/16/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>Broadway</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>12/25/2020</t>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Broadway</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HKD</t>
+          <t>Broadway</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>08/17/2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Holiday Ccy</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Holiday Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>08/17/2026</t>
         </is>
       </c>
     </row>

</xml_diff>